<commit_message>
Widen Dashboard columns so 'Facebook Marketplace' isn't cut off
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JPzyNUAq84BJUgu9eRds5E
</commit_message>
<xml_diff>
--- a/product/ProfitTrack_Reseller_Profit_Tracker.xlsx
+++ b/product/ProfitTrack_Reseller_Profit_Tracker.xlsx
@@ -1943,11 +1943,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="50322898"/>
-        <c:axId val="52129572"/>
+        <c:axId val="78834214"/>
+        <c:axId val="41096488"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="50322898"/>
+        <c:axId val="78834214"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1979,7 +1979,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52129572"/>
+        <c:crossAx val="41096488"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1987,7 +1987,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="52129572"/>
+        <c:axId val="41096488"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2053,7 +2053,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50322898"/>
+        <c:crossAx val="78834214"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2430,11 +2430,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="74266035"/>
-        <c:axId val="80117838"/>
+        <c:axId val="13380307"/>
+        <c:axId val="61701301"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="74266035"/>
+        <c:axId val="13380307"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2466,7 +2466,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80117838"/>
+        <c:crossAx val="61701301"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2474,7 +2474,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="80117838"/>
+        <c:axId val="61701301"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2550,7 +2550,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="74266035"/>
+        <c:crossAx val="13380307"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2623,7 +2623,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="8756640" y="2438280"/>
+        <a:off x="9734400" y="2438280"/>
         <a:ext cx="5939640" cy="2123640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -2653,7 +2653,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="8756640" y="4724280"/>
+        <a:off x="9734400" y="4724280"/>
         <a:ext cx="5939640" cy="2879640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -3499,13 +3499,13 @@
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="21"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="16"/>

</xml_diff>

<commit_message>
Fix chart labels and legend in iPhone preview
- Round chart source values to cents and use a single-section money
  format so previews show $486.93 instead of 486.934
- One-line series names and legend on top so it no longer overlaps
- Totals computed directly so they match the KPI to the cent

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JPzyNUAq84BJUgu9eRds5E
</commit_message>
<xml_diff>
--- a/product/ProfitTrack_Reseller_Profit_Tracker.xlsx
+++ b/product/ProfitTrack_Reseller_Profit_Tracker.xlsx
@@ -836,7 +836,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="14">
+  <numFmts count="15">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0;[RED]&quot;-$&quot;#,##0;\-"/>
     <numFmt numFmtId="166" formatCode="0.0%;[RED]\-0.0%;\-"/>
@@ -845,12 +845,13 @@
     <numFmt numFmtId="169" formatCode="\$#,##0.00&quot; avg / sale · prom / venta&quot;"/>
     <numFmt numFmtId="170" formatCode="0&quot; low-margin / margen bajo&quot;"/>
     <numFmt numFmtId="171" formatCode="General"/>
-    <numFmt numFmtId="172" formatCode="\$#,##0.00;[RED]&quot;-$&quot;#,##0.00;\-"/>
-    <numFmt numFmtId="173" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="174" formatCode="\$#,##0"/>
-    <numFmt numFmtId="175" formatCode="0.00%"/>
-    <numFmt numFmtId="176" formatCode="0%"/>
-    <numFmt numFmtId="177" formatCode="0%;[RED]\-0%;\-"/>
+    <numFmt numFmtId="172" formatCode="\$#,##0.00"/>
+    <numFmt numFmtId="173" formatCode="\$#,##0.00;[RED]&quot;-$&quot;#,##0.00;\-"/>
+    <numFmt numFmtId="174" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="175" formatCode="\$#,##0"/>
+    <numFmt numFmtId="176" formatCode="0.00%"/>
+    <numFmt numFmtId="177" formatCode="0%"/>
+    <numFmt numFmtId="178" formatCode="0%;[RED]\-0%;\-"/>
   </numFmts>
   <fonts count="37">
     <font>
@@ -1418,7 +1419,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="21" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="21" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1450,11 +1451,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="23" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="23" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="28" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="28" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1462,11 +1463,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="23" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="23" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="28" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="28" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1478,19 +1479,19 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="34" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="34" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="34" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="34" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="175" fontId="34" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="176" fontId="34" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="23" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="23" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1506,7 +1507,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="176" fontId="26" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="177" fontId="26" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1514,11 +1515,11 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="26" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="26" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="177" fontId="23" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="178" fontId="23" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1920,10 +1921,10 @@
             <c:numRef>
               <c:f>Dashboard!$F$13:$F$17</c:f>
               <c:numCache>
-                <c:formatCode>\$#,##0.00;[RED]"-$"#,##0.00;\-</c:formatCode>
+                <c:formatCode>\$#,##0.00</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>486.933825</c:v>
+                  <c:v>486.93</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>162.5</c:v>
@@ -1943,11 +1944,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="78834214"/>
-        <c:axId val="41096488"/>
+        <c:axId val="92070150"/>
+        <c:axId val="56880897"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="78834214"/>
+        <c:axId val="92070150"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1979,7 +1980,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="41096488"/>
+        <c:crossAx val="56880897"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1987,7 +1988,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="41096488"/>
+        <c:axId val="56880897"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2053,7 +2054,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78834214"/>
+        <c:crossAx val="92070150"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2130,12 +2131,11 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Dashboard!F23</c:f>
+              <c:f>"Profit / Ganancia"</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Profit
-Ganancia</c:v>
+                  <c:v>Profit / Ganancia</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2233,34 +2233,34 @@
             <c:numRef>
               <c:f>Dashboard!$F$24:$F$35</c:f>
               <c:numCache>
-                <c:formatCode>\$#,##0.00;[RED]"-$"#,##0.00;\-</c:formatCode>
+                <c:formatCode>\$#,##0.00</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>73.616325</c:v>
+                  <c:v>73.62</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>81.31</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>307.1325</c:v>
+                  <c:v>307.13</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>140.275</c:v>
+                  <c:v>140.28</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>32.165</c:v>
+                  <c:v>32.17</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>81.175</c:v>
+                  <c:v>81.18</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>85.4125</c:v>
+                  <c:v>85.41</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>125.175</c:v>
+                  <c:v>125.18</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>38.1125</c:v>
+                  <c:v>38.11</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -2281,12 +2281,11 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Dashboard!E23</c:f>
+              <c:f>"Revenue / Ingresos"</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Revenue
-Ingresos</c:v>
+                  <c:v>Revenue / Ingresos</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2379,7 +2378,7 @@
             <c:numRef>
               <c:f>Dashboard!$E$24:$E$35</c:f>
               <c:numCache>
-                <c:formatCode>\$#,##0.00;[RED]"-$"#,##0.00;\-</c:formatCode>
+                <c:formatCode>\$#,##0.00</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
                   <c:v>134.99</c:v>
@@ -2430,11 +2429,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="13380307"/>
-        <c:axId val="61701301"/>
+        <c:axId val="92772432"/>
+        <c:axId val="32581574"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="13380307"/>
+        <c:axId val="92772432"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2466,7 +2465,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61701301"/>
+        <c:crossAx val="32581574"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2474,7 +2473,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="61701301"/>
+        <c:axId val="32581574"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2550,7 +2549,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="13380307"/>
+        <c:crossAx val="92772432"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2562,7 +2561,7 @@
       </c:spPr>
     </c:plotArea>
     <c:legend>
-      <c:legendPos val="b"/>
+      <c:legendPos val="t"/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -3701,16 +3700,16 @@
       </c>
       <c r="D13" s="30"/>
       <c r="E13" s="31" t="n">
-        <f aca="false">SUMIFS(Tracker!$G$6:$G$505,Tracker!$Q$6:$Q$505,1,Tracker!$C$6:$C$505,$B13)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$G$6:$G$505,Tracker!$Q$6:$Q$505,1,Tracker!$C$6:$C$505,$B13),2)</f>
         <v>1430.99</v>
       </c>
       <c r="F13" s="31" t="n">
-        <f aca="false">SUMIFS(Tracker!$L$6:$L$505,Tracker!$Q$6:$Q$505,1,Tracker!$C$6:$C$505,$B13)</f>
-        <v>486.933825</v>
+        <f aca="false">ROUND(SUMIFS(Tracker!$L$6:$L$505,Tracker!$Q$6:$Q$505,1,Tracker!$C$6:$C$505,$B13),2)</f>
+        <v>486.93</v>
       </c>
       <c r="H13" s="32" t="n">
         <f aca="false">IF(E13=0,0,F13/E13)</f>
-        <v>0.340277587544288</v>
+        <v>0.340274914569634</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3723,11 +3722,11 @@
       </c>
       <c r="D14" s="34"/>
       <c r="E14" s="35" t="n">
-        <f aca="false">SUMIFS(Tracker!$G$6:$G$505,Tracker!$Q$6:$Q$505,1,Tracker!$C$6:$C$505,$B14)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$G$6:$G$505,Tracker!$Q$6:$Q$505,1,Tracker!$C$6:$C$505,$B14),2)</f>
         <v>300</v>
       </c>
       <c r="F14" s="35" t="n">
-        <f aca="false">SUMIFS(Tracker!$L$6:$L$505,Tracker!$Q$6:$Q$505,1,Tracker!$C$6:$C$505,$B14)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$L$6:$L$505,Tracker!$Q$6:$Q$505,1,Tracker!$C$6:$C$505,$B14),2)</f>
         <v>162.5</v>
       </c>
       <c r="H14" s="36" t="n">
@@ -3745,11 +3744,11 @@
       </c>
       <c r="D15" s="30"/>
       <c r="E15" s="31" t="n">
-        <f aca="false">SUMIFS(Tracker!$G$6:$G$505,Tracker!$Q$6:$Q$505,1,Tracker!$C$6:$C$505,$B15)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$G$6:$G$505,Tracker!$Q$6:$Q$505,1,Tracker!$C$6:$C$505,$B15),2)</f>
         <v>198</v>
       </c>
       <c r="F15" s="31" t="n">
-        <f aca="false">SUMIFS(Tracker!$L$6:$L$505,Tracker!$Q$6:$Q$505,1,Tracker!$C$6:$C$505,$B15)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$L$6:$L$505,Tracker!$Q$6:$Q$505,1,Tracker!$C$6:$C$505,$B15),2)</f>
         <v>124.44</v>
       </c>
       <c r="H15" s="32" t="n">
@@ -3767,11 +3766,11 @@
       </c>
       <c r="D16" s="34"/>
       <c r="E16" s="35" t="n">
-        <f aca="false">SUMIFS(Tracker!$G$6:$G$505,Tracker!$Q$6:$Q$505,1,Tracker!$C$6:$C$505,$B16)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$G$6:$G$505,Tracker!$Q$6:$Q$505,1,Tracker!$C$6:$C$505,$B16),2)</f>
         <v>309</v>
       </c>
       <c r="F16" s="35" t="n">
-        <f aca="false">SUMIFS(Tracker!$L$6:$L$505,Tracker!$Q$6:$Q$505,1,Tracker!$C$6:$C$505,$B16)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$L$6:$L$505,Tracker!$Q$6:$Q$505,1,Tracker!$C$6:$C$505,$B16),2)</f>
         <v>189.2</v>
       </c>
       <c r="H16" s="36" t="n">
@@ -3789,11 +3788,11 @@
       </c>
       <c r="D17" s="30"/>
       <c r="E17" s="31" t="n">
-        <f aca="false">SUMIFS(Tracker!$G$6:$G$505,Tracker!$Q$6:$Q$505,1,Tracker!$C$6:$C$505,$B17)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$G$6:$G$505,Tracker!$Q$6:$Q$505,1,Tracker!$C$6:$C$505,$B17),2)</f>
         <v>22</v>
       </c>
       <c r="F17" s="31" t="n">
-        <f aca="false">SUMIFS(Tracker!$L$6:$L$505,Tracker!$Q$6:$Q$505,1,Tracker!$C$6:$C$505,$B17)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$L$6:$L$505,Tracker!$Q$6:$Q$505,1,Tracker!$C$6:$C$505,$B17),2)</f>
         <v>1.3</v>
       </c>
       <c r="H17" s="32" t="n">
@@ -3811,16 +3810,16 @@
       </c>
       <c r="D18" s="38"/>
       <c r="E18" s="39" t="n">
-        <f aca="false">SUM(E13:E17)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$G$6:$G$505,Tracker!$Q$6:$Q$505,1),2)</f>
         <v>2259.99</v>
       </c>
       <c r="F18" s="39" t="n">
-        <f aca="false">SUM(F13:F17)</f>
-        <v>964.373825</v>
+        <f aca="false">ROUND(SUMIFS(Tracker!$L$6:$L$505,Tracker!$Q$6:$Q$505,1),2)</f>
+        <v>964.37</v>
       </c>
       <c r="H18" s="40" t="n">
         <f aca="false">IF(E18=0,0,F18/E18)</f>
-        <v>0.426715969982168</v>
+        <v>0.426714277496803</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3882,16 +3881,16 @@
       </c>
       <c r="D24" s="30"/>
       <c r="E24" s="31" t="n">
-        <f aca="false">SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+1)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+1),2)</f>
         <v>134.99</v>
       </c>
       <c r="F24" s="31" t="n">
-        <f aca="false">SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+1)</f>
-        <v>73.616325</v>
+        <f aca="false">ROUND(SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+1),2)</f>
+        <v>73.62</v>
       </c>
       <c r="H24" s="32" t="n">
         <f aca="false">IF(E24=0,0,F24/E24)</f>
-        <v>0.545346507148678</v>
+        <v>0.54537373138751</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3904,11 +3903,11 @@
       </c>
       <c r="D25" s="34"/>
       <c r="E25" s="35" t="n">
-        <f aca="false">SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+2)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+2),2)</f>
         <v>132</v>
       </c>
       <c r="F25" s="35" t="n">
-        <f aca="false">SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+2)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+2),2)</f>
         <v>81.31</v>
       </c>
       <c r="H25" s="36" t="n">
@@ -3926,16 +3925,16 @@
       </c>
       <c r="D26" s="30"/>
       <c r="E26" s="31" t="n">
-        <f aca="false">SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+3)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+3),2)</f>
         <v>979</v>
       </c>
       <c r="F26" s="31" t="n">
-        <f aca="false">SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+3)</f>
-        <v>307.1325</v>
+        <f aca="false">ROUND(SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+3),2)</f>
+        <v>307.13</v>
       </c>
       <c r="H26" s="32" t="n">
         <f aca="false">IF(E26=0,0,F26/E26)</f>
-        <v>0.313720633299285</v>
+        <v>0.313718079673136</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3948,16 +3947,16 @@
       </c>
       <c r="D27" s="34"/>
       <c r="E27" s="35" t="n">
-        <f aca="false">SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+4)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+4),2)</f>
         <v>205</v>
       </c>
       <c r="F27" s="35" t="n">
-        <f aca="false">SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+4)</f>
-        <v>140.275</v>
+        <f aca="false">ROUND(SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+4),2)</f>
+        <v>140.28</v>
       </c>
       <c r="H27" s="36" t="n">
         <f aca="false">IF(E27=0,0,F27/E27)</f>
-        <v>0.684268292682927</v>
+        <v>0.684292682926829</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3970,16 +3969,16 @@
       </c>
       <c r="D28" s="30"/>
       <c r="E28" s="31" t="n">
-        <f aca="false">SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+5)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+5),2)</f>
         <v>86</v>
       </c>
       <c r="F28" s="31" t="n">
-        <f aca="false">SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+5)</f>
-        <v>32.165</v>
+        <f aca="false">ROUND(SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+5),2)</f>
+        <v>32.17</v>
       </c>
       <c r="H28" s="32" t="n">
         <f aca="false">IF(E28=0,0,F28/E28)</f>
-        <v>0.374011627906977</v>
+        <v>0.374069767441861</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3992,16 +3991,16 @@
       </c>
       <c r="D29" s="34"/>
       <c r="E29" s="35" t="n">
-        <f aca="false">SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+6)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+6),2)</f>
         <v>195</v>
       </c>
       <c r="F29" s="35" t="n">
-        <f aca="false">SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+6)</f>
-        <v>81.175</v>
+        <f aca="false">ROUND(SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+6),2)</f>
+        <v>81.18</v>
       </c>
       <c r="H29" s="36" t="n">
         <f aca="false">IF(E29=0,0,F29/E29)</f>
-        <v>0.416282051282051</v>
+        <v>0.416307692307692</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4014,16 +4013,16 @@
       </c>
       <c r="D30" s="30"/>
       <c r="E30" s="31" t="n">
-        <f aca="false">SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+7)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+7),2)</f>
         <v>157</v>
       </c>
       <c r="F30" s="31" t="n">
-        <f aca="false">SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+7)</f>
-        <v>85.4125</v>
+        <f aca="false">ROUND(SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+7),2)</f>
+        <v>85.41</v>
       </c>
       <c r="H30" s="32" t="n">
         <f aca="false">IF(E30=0,0,F30/E30)</f>
-        <v>0.544028662420382</v>
+        <v>0.544012738853503</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4036,16 +4035,16 @@
       </c>
       <c r="D31" s="34"/>
       <c r="E31" s="35" t="n">
-        <f aca="false">SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+8)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+8),2)</f>
         <v>210</v>
       </c>
       <c r="F31" s="35" t="n">
-        <f aca="false">SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+8)</f>
-        <v>125.175</v>
+        <f aca="false">ROUND(SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+8),2)</f>
+        <v>125.18</v>
       </c>
       <c r="H31" s="36" t="n">
         <f aca="false">IF(E31=0,0,F31/E31)</f>
-        <v>0.596071428571429</v>
+        <v>0.596095238095238</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4058,16 +4057,16 @@
       </c>
       <c r="D32" s="30"/>
       <c r="E32" s="31" t="n">
-        <f aca="false">SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+9)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+9),2)</f>
         <v>161</v>
       </c>
       <c r="F32" s="31" t="n">
-        <f aca="false">SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+9)</f>
-        <v>38.1125</v>
+        <f aca="false">ROUND(SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+9),2)</f>
+        <v>38.11</v>
       </c>
       <c r="H32" s="32" t="n">
         <f aca="false">IF(E32=0,0,F32/E32)</f>
-        <v>0.236723602484472</v>
+        <v>0.236708074534161</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4080,11 +4079,11 @@
       </c>
       <c r="D33" s="34"/>
       <c r="E33" s="35" t="n">
-        <f aca="false">SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+10)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+10),2)</f>
         <v>0</v>
       </c>
       <c r="F33" s="35" t="n">
-        <f aca="false">SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+10)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+10),2)</f>
         <v>0</v>
       </c>
       <c r="H33" s="36" t="n">
@@ -4102,11 +4101,11 @@
       </c>
       <c r="D34" s="30"/>
       <c r="E34" s="31" t="n">
-        <f aca="false">SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+11)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+11),2)</f>
         <v>0</v>
       </c>
       <c r="F34" s="31" t="n">
-        <f aca="false">SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+11)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+11),2)</f>
         <v>0</v>
       </c>
       <c r="H34" s="32" t="n">
@@ -4124,11 +4123,11 @@
       </c>
       <c r="D35" s="34"/>
       <c r="E35" s="35" t="n">
-        <f aca="false">SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+12)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,$C$22*100+12),2)</f>
         <v>0</v>
       </c>
       <c r="F35" s="35" t="n">
-        <f aca="false">SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+12)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,$C$22*100+12),2)</f>
         <v>0</v>
       </c>
       <c r="H35" s="36" t="n">
@@ -4146,16 +4145,16 @@
       </c>
       <c r="D36" s="38"/>
       <c r="E36" s="39" t="n">
-        <f aca="false">SUM(E24:E35)</f>
+        <f aca="false">ROUND(SUMIFS(Tracker!$G$6:$G$505,Tracker!$R$6:$R$505,"&gt;="&amp;($C$22*100+1),Tracker!$R$6:$R$505,"&lt;="&amp;($C$22*100+12)),2)</f>
         <v>2259.99</v>
       </c>
       <c r="F36" s="39" t="n">
-        <f aca="false">SUM(F24:F35)</f>
-        <v>964.373825</v>
+        <f aca="false">ROUND(SUMIFS(Tracker!$L$6:$L$505,Tracker!$R$6:$R$505,"&gt;="&amp;($C$22*100+1),Tracker!$R$6:$R$505,"&lt;="&amp;($C$22*100+12)),2)</f>
+        <v>964.37</v>
       </c>
       <c r="H36" s="40" t="n">
         <f aca="false">IF(E36=0,0,F36/E36)</f>
-        <v>0.426715969982168</v>
+        <v>0.426714277496803</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Lock Dashboard so its formulas can't be overwritten
Sheet protection without a password; only the Year cell stays
editable. Guide step 7 and FAQ explain how to unlock.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JPzyNUAq84BJUgu9eRds5E
</commit_message>
<xml_diff>
--- a/product/ProfitTrack_Reseller_Profit_Tracker.xlsx
+++ b/product/ProfitTrack_Reseller_Profit_Tracker.xlsx
@@ -187,7 +187,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="204">
   <si>
     <t xml:space="preserve">RESELLER TOOLKIT  •  KIT PARA REVENDEDORES</t>
   </si>
@@ -697,10 +697,10 @@
     <t xml:space="preserve">Si un artículo se devuelve, cambia el Estado a 'Returned / Devuelto'. Se queda en tu registro (en gris) pero se excluye de todos los números del Panel.</t>
   </si>
   <si>
-    <t xml:space="preserve">Open the Dashboard to see your KPIs, profit by platform, the monthly trend chart and your Top 5 sales. Everything updates instantly. Change the yellow Year cell to view another year.</t>
+    <t xml:space="preserve">Open the Dashboard to see your KPIs, profit by platform, the monthly trend chart and your Top 5 sales. Everything updates instantly. The Dashboard is locked to protect its formulas – only the yellow Year cell can be changed.</t>
   </si>
   <si>
-    <t xml:space="preserve">Abre el Dashboard (Panel) para ver tus indicadores, ganancia por plataforma, la gráfica mensual y tus Top 5 ventas. Todo se actualiza al instante. Cambia la celda amarilla del Año para ver otro año.</t>
+    <t xml:space="preserve">Abre el Dashboard (Panel) para ver tus indicadores, ganancia por plataforma, la gráfica mensual y tus Top 5 ventas. Todo se actualiza al instante. El Panel está bloqueado para proteger sus fórmulas – solo se puede cambiar la celda amarilla del Año.</t>
   </si>
   <si>
     <t xml:space="preserve">BONUS — before buying inventory, use the Sourcing List. Set your minimum margin and minimum profit (yellow cells), enter the asking price and your estimated sale price, and get an instant ✔ BUY / ✖ PASS plus the Max Buy Price to negotiate with.</t>
@@ -803,6 +803,12 @@
   </si>
   <si>
     <t xml:space="preserve">P: Una venta no muestra ganancia.  R: La ganancia aparece cuando llenas el Nombre del Producto y el Precio de Venta.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q: Why can't I type on the Dashboard?  A: It's locked so its formulas can't be erased by accident – add or change sales on the Tracker instead. Only the yellow Year cell is editable. To unlock (no password): Excel → Review → Unprotect Sheet; Google Sheets → Data → Protect sheets and ranges.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P: ¿Por qué no puedo escribir en el Panel?  R: Está bloqueado para que sus fórmulas no se borren por accidente – agrega o cambia ventas en el Tracker. Solo la celda amarilla del Año se puede editar. Para desbloquear (sin contraseña): Excel → Revisar → Desproteger hoja; Google Sheets → Datos → Proteger hojas y rangos.</t>
   </si>
   <si>
     <t xml:space="preserve">Phone, Tablet &amp; Computer  /  Celular, Tableta y Computadora</t>
@@ -1435,9 +1441,9 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="26" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="26" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+      <protection locked="false" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
@@ -1944,11 +1950,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="92070150"/>
-        <c:axId val="56880897"/>
+        <c:axId val="36785636"/>
+        <c:axId val="63978515"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="92070150"/>
+        <c:axId val="36785636"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1980,7 +1986,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="56880897"/>
+        <c:crossAx val="63978515"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1988,7 +1994,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="56880897"/>
+        <c:axId val="63978515"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2054,7 +2060,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="92070150"/>
+        <c:crossAx val="36785636"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2429,11 +2435,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="92772432"/>
-        <c:axId val="32581574"/>
+        <c:axId val="33268885"/>
+        <c:axId val="83061632"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="92772432"/>
+        <c:axId val="33268885"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2465,7 +2471,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="32581574"/>
+        <c:crossAx val="83061632"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2473,7 +2479,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="32581574"/>
+        <c:axId val="83061632"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2549,7 +2555,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="92772432"/>
+        <c:crossAx val="33268885"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3491,7 +3497,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF14B8A6"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:N46"/>
@@ -4353,6 +4358,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="true"/>
   <mergeCells count="56">
     <mergeCell ref="B1:N1"/>
     <mergeCell ref="B2:N2"/>
@@ -30992,7 +30998,7 @@
     <tabColor rgb="FF0B1F3A"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.5"/>
@@ -31112,7 +31118,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="81" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="65" t="n">
         <v>7</v>
       </c>
@@ -31289,22 +31295,22 @@
         <v>192</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="68" t="s">
+    <row r="36" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C36" s="73" t="s">
         <v>193</v>
       </c>
-      <c r="C37" s="68"/>
-      <c r="D37" s="68"/>
-    </row>
-    <row r="38" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C38" s="73" t="s">
+      <c r="D36" s="73" t="s">
         <v>194</v>
       </c>
-      <c r="D38" s="73" t="s">
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="68" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="39" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C38" s="68"/>
+      <c r="D38" s="68"/>
+    </row>
+    <row r="39" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C39" s="73" t="s">
         <v>196</v>
       </c>
@@ -31312,7 +31318,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C40" s="73" t="s">
         <v>198</v>
       </c>
@@ -31320,12 +31326,20 @@
         <v>199</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C41" s="73" t="s">
         <v>200</v>
       </c>
       <c r="D41" s="73" t="s">
         <v>201</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C42" s="73" t="s">
+        <v>202</v>
+      </c>
+      <c r="D42" s="73" t="s">
+        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -31337,7 +31351,7 @@
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="B30:D30"/>
     <mergeCell ref="B32:D32"/>
-    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="B38:D38"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Taller headers and wider number columns for phone screens
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JPzyNUAq84BJUgu9eRds5E
</commit_message>
<xml_diff>
--- a/product/ProfitTrack_Reseller_Profit_Tracker.xlsx
+++ b/product/ProfitTrack_Reseller_Profit_Tracker.xlsx
@@ -1950,11 +1950,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="36785636"/>
-        <c:axId val="63978515"/>
+        <c:axId val="80958483"/>
+        <c:axId val="94612046"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="36785636"/>
+        <c:axId val="80958483"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1986,7 +1986,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="63978515"/>
+        <c:crossAx val="94612046"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1994,7 +1994,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="63978515"/>
+        <c:axId val="94612046"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2060,7 +2060,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36785636"/>
+        <c:crossAx val="80958483"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2435,11 +2435,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="33268885"/>
-        <c:axId val="83061632"/>
+        <c:axId val="59227558"/>
+        <c:axId val="83053252"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="33268885"/>
+        <c:axId val="59227558"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2471,7 +2471,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83061632"/>
+        <c:crossAx val="83053252"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2479,7 +2479,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="83061632"/>
+        <c:axId val="83053252"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2555,7 +2555,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="33268885"/>
+        <c:crossAx val="59227558"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4441,12 +4441,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="4" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="4" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="26"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="19" min="16" style="0" width="13"/>
@@ -4526,7 +4521,7 @@
       <c r="N4" s="7"/>
       <c r="O4" s="7"/>
     </row>
-    <row r="5" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="27" t="s">
         <v>66</v>
       </c>
@@ -27054,13 +27049,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="14"/>
@@ -27202,7 +27195,7 @@
       <c r="P8" s="62"/>
       <c r="Q8" s="62"/>
     </row>
-    <row r="10" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="27" t="s">
         <v>114</v>
       </c>

</xml_diff>